<commit_message>
bug fixes after code rewiev_6
</commit_message>
<xml_diff>
--- a/data/raw/test_articles.xlsx
+++ b/data/raw/test_articles.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20827"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0C53E0F-105E-4946-8764-0BB1C3427857}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86B66E8C-A17A-41E6-B744-F7AC6333D997}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,12 +23,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
   <si>
-    <t>Артикул</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
+    <t>артикул</t>
   </si>
 </sst>
 </file>
@@ -134,7 +131,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -413,115 +410,115 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A22"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>1000100310</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>1000100311</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3">
         <v>1009806735</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="4">
         <v>1009806733</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="4">
         <v>1009806734</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="4">
         <v>1010601542</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="4">
         <v>1009806741</v>
       </c>
     </row>
-    <row r="9" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="4">
         <v>1010600689</v>
       </c>
     </row>
-    <row r="10" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="4">
         <v>1991100323</v>
       </c>
     </row>
-    <row r="11" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="4">
         <v>1000400196</v>
       </c>
     </row>
-    <row r="12" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="4">
         <v>1000400458</v>
       </c>
     </row>
-    <row r="13" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="4">
         <v>1000000876</v>
       </c>
     </row>
-    <row r="14" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="4">
         <v>1009900947</v>
       </c>
     </row>
-    <row r="15" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="4">
         <v>1000400428</v>
       </c>
     </row>
-    <row r="16" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="4">
         <v>1000300679</v>
       </c>
     </row>
-    <row r="17" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="4">
         <v>1010601571</v>
       </c>
     </row>
-    <row r="18" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="4">
         <v>1019902592</v>
       </c>
     </row>
-    <row r="19" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="4">
         <v>1019902593</v>
       </c>
     </row>
-    <row r="20" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="4">
         <v>1010601865</v>
       </c>
     </row>
-    <row r="21" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="5">
         <v>1010601507</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A22">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: correct sales calculation, optimize report loading, fix forecasting progress bar
</commit_message>
<xml_diff>
--- a/data/raw/test_articles.xlsx
+++ b/data/raw/test_articles.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A628E1A8-8082-4429-A1A3-883AA7C17445}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E52AC8C-3FF1-437B-BF18-7D5F12BA5EA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,9 +23,27 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>артикул</t>
+  </si>
+  <si>
+    <t>203020003249</t>
+  </si>
+  <si>
+    <t>0445120134</t>
+  </si>
+  <si>
+    <t>1110100317</t>
+  </si>
+  <si>
+    <t>1022099027</t>
+  </si>
+  <si>
+    <t>605110000754</t>
+  </si>
+  <si>
+    <t>1020521445</t>
   </si>
 </sst>
 </file>
@@ -41,16 +59,19 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -61,7 +82,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -69,72 +90,25 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -412,127 +386,75 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A24"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:A13"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="12.90625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="1">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A3" s="3">
+        <v>1009806733</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A7" s="4">
+        <v>1020201963</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A8" s="4">
+        <v>450010294</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A9" s="4">
+        <v>1010306624</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A12" s="3">
         <v>1000100310</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" s="2">
-        <v>1000100311</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="3">
-        <v>1009806735</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="4">
-        <v>1009806733</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="4">
-        <v>1009806734</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="4">
-        <v>1010601542</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="4">
-        <v>1009806741</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="4">
-        <v>1010600689</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="4">
-        <v>1991100323</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="4">
-        <v>1000400196</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="4">
-        <v>1000400458</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="4">
-        <v>1000000876</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="4">
-        <v>1009900947</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="4">
-        <v>1000400428</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="4">
-        <v>1000300679</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="4">
-        <v>1010601571</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="4">
-        <v>1019902592</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="4">
-        <v>1019902593</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="4">
-        <v>1010601865</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="5">
-        <v>1010601507</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A22">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A23" s="6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A24" s="6">
-        <v>1</v>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A13" s="3">
+        <v>93200043</v>
       </c>
     </row>
   </sheetData>

</xml_diff>